<commit_message>
1.1 - data_files and analyses updated
</commit_message>
<xml_diff>
--- a/docs/data_dictionary.xlsx
+++ b/docs/data_dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e62e7c97e835051/Altieri/Estudos/Sistemas/Plano Carreira/Bases Hashtag - Treinamentos/11. Aula Claude/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_ADF5BE0B1262A03EE10600744D5DCE3AE7CC7620" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C23463D1-4F7C-4E01-8B7D-8E7E3757BE60}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="11_ADF5BE0B1262A03EE10600744D5DCE3AE7CC7620" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66E298F6-7FFE-43DE-91F8-BDD74F30DFB9}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="5760" yWindow="3720" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Dictionary" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data Dictionary'!$A$4:$G$62</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1234,7 +1247,7 @@
       <c r="G14" s="6"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="9" t="s">
         <v>46</v>
       </c>
       <c r="B15" s="5" t="s">
@@ -1257,7 +1270,7 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="8" t="s">
         <v>46</v>
       </c>
       <c r="B16" s="5" t="s">
@@ -1410,7 +1423,7 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="8" t="s">
         <v>59</v>
       </c>
       <c r="B23" s="5" t="s">
@@ -1431,7 +1444,7 @@
       <c r="G23" s="6"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="8" t="s">
         <v>59</v>
       </c>
       <c r="B24" s="5" t="s">
@@ -1452,7 +1465,7 @@
       <c r="G24" s="6"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="8" t="s">
         <v>59</v>
       </c>
       <c r="B25" s="5" t="s">
@@ -1473,7 +1486,7 @@
       <c r="G25" s="6"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="9" t="s">
         <v>59</v>
       </c>
       <c r="B26" s="5" t="s">

</xml_diff>

<commit_message>
chore: ignore internal docs (handoff, passo_a_passo)
</commit_message>
<xml_diff>
--- a/docs/data_dictionary.xlsx
+++ b/docs/data_dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e62e7c97e835051/Altieri/Estudos/Sistemas/Plano Carreira/Bases Hashtag - Treinamentos/11. Aula Claude/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="11_ADF5BE0B1262A03EE10600744D5DCE3AE7CC7620" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66E298F6-7FFE-43DE-91F8-BDD74F30DFB9}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="11_ADF5BE0B1262A03EE10600744D5DCE3AE7CC7620" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC90B922-2AD6-4739-84B3-EEA692A1C4E5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1291,7 +1291,7 @@
       <c r="G16" s="6"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="9" t="s">
         <v>46</v>
       </c>
       <c r="B17" s="5" t="s">
@@ -1312,7 +1312,7 @@
       <c r="G17" s="6"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="8" t="s">
         <v>46</v>
       </c>
       <c r="B18" s="5" t="s">
@@ -1333,7 +1333,7 @@
       <c r="G18" s="6"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="9" t="s">
         <v>46</v>
       </c>
       <c r="B19" s="5" t="s">
@@ -1677,7 +1677,7 @@
       <c r="G34" s="6"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="9" t="s">
         <v>99</v>
       </c>
       <c r="B35" s="5" t="s">
@@ -1700,7 +1700,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="8" t="s">
         <v>99</v>
       </c>
       <c r="B36" s="5" t="s">
@@ -1721,7 +1721,7 @@
       <c r="G36" s="6"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="9" t="s">
         <v>99</v>
       </c>
       <c r="B37" s="5" t="s">

</xml_diff>